<commit_message>
Picking sheet: re-match choker and sunglasses on CJ after photo check; price the owner's three picks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kalo_cj/picking_sheet_2026-10-29.xlsx
+++ b/data/kalo_cj/picking_sheet_2026-10-29.xlsx
@@ -652,44 +652,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>A11</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Shoes</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Clarks Collection Loafers -Westlynn Ayla</t>
+          <t>The Barb Wire Choker Danielle Guizio X The M Jewelers Necklace</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>204227.68</v>
+        <v>87038.5</v>
       </c>
       <c r="F2" t="n">
-        <v>3112</v>
+        <v>1238</v>
       </c>
       <c r="G2" t="n">
-        <v>65.63</v>
+        <v>70.31</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>97.41</t>
+          <t>-10.01</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>QVC, Inc</t>
+          <t>themjewelersny</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/view/product/1731966485847774151?region=US</t>
+          <t>https://www.tiktok.com/view/product/1732377057880544126?region=US</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -699,34 +699,34 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>match</t>
+          <t>partial</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Same chunky lug-sole penny loafer shape in black and brown; CJ has a metal bit instead of the croc-embossed strap.</t>
+          <t>Re-matched: CJLX1504225 thin barbed-wire choker, same shape as the winner but silver not gold. Photo tag reads ORNAMENTUS (possible other brand): sample first, don't reuse that photo.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Women Classic Elegant Fashion 2026 New Round Toe Block Low Heel Loafer Leather Shoes Elegant Versatile Pumps</t>
+          <t>Barbed Wire Necklace</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>CJNS3043308</t>
+          <t>CJLX1504225</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>https://www.cjdropshipping.com/product/women-classic-elegant-fashion-2026-new-round-toe-block-low-heel-loafer-leather-shoes-elegant-versatile-pumps-p-2085598370886311938.html</t>
+          <t>https://www.cjdropshipping.com/product/barbed-wire-necklace-p-1537624790973034496.html</t>
         </is>
       </c>
       <c r="Q2" t="n">
-        <v>6.6</v>
+        <v>6.29</v>
       </c>
       <c r="R2" t="n">
-        <v>500</v>
+        <v>24</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -734,11 +734,11 @@
         </is>
       </c>
       <c r="T2" t="n">
-        <v>11.32</v>
+        <v>4.82</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>LuWei Ordinary US</t>
+          <t>CJPacket Super Pure Electricity</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -747,82 +747,79 @@
         </is>
       </c>
       <c r="W2" t="n">
-        <v>17.92</v>
+        <v>11.11</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>22.23</v>
+        <v>33.35</v>
       </c>
       <c r="Y2" t="n">
-        <v>42.23</v>
+        <v>53.35</v>
       </c>
       <c r="Z2" t="n">
-        <v>52.99</v>
+        <v>44.99</v>
       </c>
       <c r="AA2" t="n">
-        <v>-19</v>
+        <v>-36</v>
       </c>
       <c r="AB2" t="b">
         <v>1</v>
       </c>
       <c r="AC2" t="n">
-        <v>5</v>
+        <v>70</v>
       </c>
       <c r="AD2" t="n">
-        <v>103466</v>
+        <v>95350</v>
       </c>
       <c r="AE2" t="n">
         <v>0</v>
       </c>
-      <c r="AF2" t="n">
-        <v>0</v>
-      </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>Generic round-toe low block-heel loafer in black/brown PU, unbranded lookalike of the Clarks heeled loafer (no Clarks leather or cushioning); low listedNum (5).</t>
+          <t>Re-matched after photo check: thin barbed-wire choker, same shape as the winner but silver only (no gold on CJ). Clasp tag in CJ photo reads ORNAMENTUS (another brand?): sample before listing.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C08</t>
+          <t>S12</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Clothing</t>
+          <t>Shoes</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>April Satin Pant</t>
+          <t>Clarks Collection Loafers -Westlynn Ayla</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>424640.14</v>
+        <v>204227.68</v>
       </c>
       <c r="F3" t="n">
-        <v>6921</v>
+        <v>3112</v>
       </c>
       <c r="G3" t="n">
-        <v>61.36</v>
+        <v>65.63</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>48.81</t>
+          <t>97.41</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>April Seven Studio</t>
+          <t>QVC, Inc</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/view/product/1731468041024738009?region=US</t>
+          <t>https://www.tiktok.com/view/product/1731966485847774151?region=US</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -837,29 +834,29 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Same high-waist satin wide-leg pant; CJ photo is pink but black is a variant. Fabric is acetate satin.</t>
+          <t>Same chunky lug-sole penny loafer shape in black and brown; CJ has a metal bit instead of the croc-embossed strap.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Casual Pants High Waist Acetate Satin Wide Leg Pants For Women</t>
+          <t>Women Classic Elegant Fashion 2026 New Round Toe Block Low Heel Loafer Leather Shoes Elegant Versatile Pumps</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>CJTZ1911661</t>
+          <t>CJNS3043308</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>https://www.cjdropshipping.com/product/casual-pants-high-waist-acetate-satin-wide-leg-pants-for-women-p-1731134489503469568.html</t>
+          <t>https://www.cjdropshipping.com/product/women-classic-elegant-fashion-2026-new-round-toe-block-low-heel-loafer-leather-shoes-elegant-versatile-pumps-p-2085598370886311938.html</t>
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>9.449999999999999</v>
+        <v>6.6</v>
       </c>
       <c r="R3" t="n">
-        <v>380</v>
+        <v>500</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -867,7 +864,7 @@
         </is>
       </c>
       <c r="T3" t="n">
-        <v>9.5</v>
+        <v>11.32</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -880,28 +877,28 @@
         </is>
       </c>
       <c r="W3" t="n">
-        <v>18.95</v>
+        <v>17.92</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>17.26</v>
+        <v>22.23</v>
       </c>
       <c r="Y3" t="n">
-        <v>37.26</v>
+        <v>42.23</v>
       </c>
       <c r="Z3" t="n">
-        <v>53.99</v>
+        <v>52.99</v>
       </c>
       <c r="AA3" t="n">
-        <v>-12</v>
+        <v>-19</v>
       </c>
       <c r="AB3" t="b">
         <v>1</v>
       </c>
       <c r="AC3" t="n">
-        <v>78</v>
+        <v>5</v>
       </c>
       <c r="AD3" t="n">
-        <v>191156</v>
+        <v>103466</v>
       </c>
       <c r="AE3" t="n">
         <v>0</v>
@@ -911,51 +908,51 @@
       </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>High-waist acetate-look satin wide-leg pants in apricot/pink/black/gray; Kalodata title gives no detail, so exact cut and waistband may differ.</t>
+          <t>Generic round-toe low block-heel loafer in black/brown PU, unbranded lookalike of the Clarks heeled loafer (no Clarks leather or cushioning); low listedNum (5).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>A02</t>
+          <t>C08</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Clothing</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>WMP Eyewear Astra Cat-Eye Sunglasses for Women, Bold Modern Frame, Lightweight Trendy Sunglasses with UV Protection</t>
+          <t>April Satin Pant</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>196556.64</v>
+        <v>424640.14</v>
       </c>
       <c r="F4" t="n">
-        <v>4328</v>
+        <v>6921</v>
       </c>
       <c r="G4" t="n">
-        <v>45.42</v>
+        <v>61.36</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>-39.88</t>
+          <t>48.81</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>WMP Eyewear</t>
+          <t>April Seven Studio</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/view/product/1732201295444087593?region=US</t>
+          <t>https://www.tiktok.com/view/product/1731468041024738009?region=US</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -965,34 +962,34 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>match</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Winner is a bold thick oval cat-eye; CJ is a thin half-rim mini cat-eye. Different look.</t>
+          <t>Same high-waist satin wide-leg pant; CJ photo is pink but black is a variant. Fabric is acetate satin.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Cat Eye Sunglasses Women European And American Fashion Trending</t>
+          <t>Casual Pants High Waist Acetate Satin Wide Leg Pants For Women</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>CJCF1968233</t>
+          <t>CJTZ1911661</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>https://www.cjdropshipping.com/product/cat-eye-sunglasses-women-european-and-american-fashion-trending-p-1757567002828349440.html</t>
+          <t>https://www.cjdropshipping.com/product/casual-pants-high-waist-acetate-satin-wide-leg-pants-for-women-p-1731134489503469568.html</t>
         </is>
       </c>
       <c r="Q4" t="n">
-        <v>1.65</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="R4" t="n">
-        <v>40</v>
+        <v>380</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -1000,7 +997,7 @@
         </is>
       </c>
       <c r="T4" t="n">
-        <v>5.27</v>
+        <v>9.5</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
@@ -1013,28 +1010,28 @@
         </is>
       </c>
       <c r="W4" t="n">
-        <v>6.92</v>
+        <v>18.95</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>14.61</v>
+        <v>17.26</v>
       </c>
       <c r="Y4" t="n">
-        <v>34.61</v>
+        <v>37.26</v>
       </c>
       <c r="Z4" t="n">
-        <v>40.99</v>
+        <v>53.99</v>
       </c>
       <c r="AA4" t="n">
-        <v>-10</v>
+        <v>-12</v>
       </c>
       <c r="AB4" t="b">
         <v>1</v>
       </c>
       <c r="AC4" t="n">
-        <v>357</v>
+        <v>78</v>
       </c>
       <c r="AD4" t="n">
-        <v>111129</v>
+        <v>191156</v>
       </c>
       <c r="AE4" t="n">
         <v>0</v>
@@ -1044,51 +1041,51 @@
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>Generic plastic-frame trendy cat-eye sunglasses in 9 colourways; frame thickness vs the bold Astra and the UV rating are not stated on the listing.</t>
+          <t>High-waist acetate-look satin wide-leg pants in apricot/pink/black/gray; Kalodata title gives no detail, so exact cut and waistband may differ.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>A02</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Clothing</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Comfrt | VIP Airplane Mode Travel Zip Hoodie - Mega | CloudTouch Fleece Zip-Up With Silk-Lined Hood &amp; Eye Mask</t>
+          <t>WMP Eyewear Astra Cat-Eye Sunglasses for Women, Bold Modern Frame, Lightweight Trendy Sunglasses with UV Protection</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>318470.2</v>
+        <v>196556.64</v>
       </c>
       <c r="F5" t="n">
-        <v>5091</v>
+        <v>4328</v>
       </c>
       <c r="G5" t="n">
-        <v>62.56</v>
+        <v>45.42</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>52.08</t>
+          <t>-39.88</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Comfrt</t>
+          <t>WMP Eyewear</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/view/product/1732607430962811779?region=US</t>
+          <t>https://www.tiktok.com/view/product/1732201295444087593?region=US</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1098,34 +1095,34 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>match</t>
+          <t>partial</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Same eye-mask hood idea (the TikTok hook); CJ is a pullover not a zip-up and has no mega-fit claim.</t>
+          <t>Re-matched: CJCF1177466 thick cat-eye in brown tortoise; bold frame like the winner but a sharper cat-eye shape and lighter colour.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Eye-mask Hoodie 350g Fleece-lined Sweatshirt</t>
+          <t>Cat-eye Frame Sunglasses INS Style Sunglasses</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>CJWY2725041</t>
+          <t>CJCF1177466</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>https://www.cjdropshipping.com/product/eye-mask-hoodie-350g-fleece-lined-sweatshirt-p-2601110708231630100.html</t>
+          <t>https://www.cjdropshipping.com/product/cat-eye-frame-sunglasses-ins-style-sunglasses-p-1405348596290818048.html</t>
         </is>
       </c>
       <c r="Q5" t="n">
-        <v>13.43</v>
+        <v>1.46</v>
       </c>
       <c r="R5" t="n">
-        <v>410</v>
+        <v>40</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -1133,7 +1130,7 @@
         </is>
       </c>
       <c r="T5" t="n">
-        <v>9.949999999999999</v>
+        <v>5.27</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
@@ -1146,82 +1143,79 @@
         </is>
       </c>
       <c r="W5" t="n">
-        <v>23.38</v>
+        <v>6.73</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>13.94</v>
+        <v>14.8</v>
       </c>
       <c r="Y5" t="n">
-        <v>33.94</v>
+        <v>34.8</v>
       </c>
       <c r="Z5" t="n">
-        <v>58.99</v>
+        <v>40.99</v>
       </c>
       <c r="AA5" t="n">
-        <v>-6</v>
+        <v>-10</v>
       </c>
       <c r="AB5" t="b">
         <v>1</v>
       </c>
       <c r="AC5" t="n">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="AD5" t="n">
-        <v>119616</v>
+        <v>86361</v>
       </c>
       <c r="AE5" t="n">
         <v>0</v>
       </c>
-      <c r="AF5" t="n">
-        <v>0</v>
-      </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>Fleece-lined hoodie with built-in eye-mask hood (same travel angle) in 4 colours; pullover not zip-up, no silk-lined hood, men's/unisex cut.</t>
+          <t>Re-matched after photo check: thick acetate-look cat-eye, brown (tortoise) variant; sharper cat-eye than the winner's soft oval. Also white and grey.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>S01</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Shoes</t>
+          <t>Clothing</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Crocs Adult Classic Cozzzy Slippers, Fuzzy Slippers</t>
+          <t>Comfrt | VIP Airplane Mode Travel Zip Hoodie - Mega | CloudTouch Fleece Zip-Up With Silk-Lined Hood &amp; Eye Mask</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>558438.3</v>
+        <v>318470.2</v>
       </c>
       <c r="F6" t="n">
-        <v>11635</v>
+        <v>5091</v>
       </c>
       <c r="G6" t="n">
-        <v>48</v>
+        <v>62.56</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2042.92</t>
+          <t>52.08</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>CROCS US SHOP</t>
+          <t>Comfrt</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/view/product/1730493404455474110?region=US</t>
+          <t>https://www.tiktok.com/view/product/1732607430962811779?region=US</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1231,34 +1225,34 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>match</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Winner is an all-fur slipper; CJ is a perforated garden clog with a fur cuff.</t>
+          <t>Same eye-mask hood idea (the TikTok hook); CJ is a pullover not a zip-up and has no mega-fit claim.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Fuzzy Plush Garden Clogs Mules Slippers Home Indoor Couple Slippers</t>
+          <t>Eye-mask Hoodie 350g Fleece-lined Sweatshirt</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>CJNS1050784</t>
+          <t>CJWY2725041</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>https://www.cjdropshipping.com/product/fuzzy-plush-garden-clogs-mules-slippers-home-indoor-couple-slippers-p-1373889976009363456.html</t>
+          <t>https://www.cjdropshipping.com/product/eye-mask-hoodie-350g-fleece-lined-sweatshirt-p-2601110708231630100.html</t>
         </is>
       </c>
       <c r="Q6" t="n">
-        <v>2.3</v>
+        <v>13.43</v>
       </c>
       <c r="R6" t="n">
-        <v>269</v>
+        <v>410</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1266,7 +1260,7 @@
         </is>
       </c>
       <c r="T6" t="n">
-        <v>7.81</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
@@ -1279,42 +1273,45 @@
         </is>
       </c>
       <c r="W6" t="n">
-        <v>10.11</v>
+        <v>23.38</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>13.8</v>
+        <v>13.94</v>
       </c>
       <c r="Y6" t="n">
-        <v>33.8</v>
+        <v>33.94</v>
       </c>
       <c r="Z6" t="n">
-        <v>43.99</v>
+        <v>58.99</v>
       </c>
       <c r="AA6" t="n">
-        <v>-8</v>
+        <v>-6</v>
       </c>
       <c r="AB6" t="b">
         <v>1</v>
       </c>
       <c r="AC6" t="n">
-        <v>543</v>
+        <v>10</v>
       </c>
       <c r="AD6" t="n">
-        <v>2000000</v>
+        <v>119616</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>0</v>
       </c>
       <c r="AF6" t="n">
         <v>0</v>
       </c>
       <c r="AI6" t="inlineStr">
         <is>
-          <t>Unbranded plush-lined garden clog mule (closed toe, fuzzy lining) rather than Crocs Cozzzy open sandal-slipper; listed as men's/couple sizes 36-45.</t>
+          <t>Fleece-lined hoodie with built-in eye-mask hood (same travel angle) in 4 colours; pullover not zip-up, no silk-lined hood, men's/unisex cut.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>S07</t>
+          <t>S01</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1323,25 +1320,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Crocs Adult Unfurgettable Furry Lined Clogs, Fuzzy Slippers</t>
+          <t>Crocs Adult Classic Cozzzy Slippers, Fuzzy Slippers</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>238816.09</v>
+        <v>558438.3</v>
       </c>
       <c r="F7" t="n">
-        <v>5002</v>
+        <v>11635</v>
       </c>
       <c r="G7" t="n">
-        <v>47.74</v>
+        <v>48</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>58.31</t>
+          <t>2042.92</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1351,7 +1348,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/view/product/1732481650106799038?region=US</t>
+          <t>https://www.tiktok.com/view/product/1730493404455474110?region=US</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1366,7 +1363,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Winner is a fur-covered clog; CJ is a perforated garden clog with a fur cuff.</t>
+          <t>Winner is an all-fur slipper; CJ is a perforated garden clog with a fur cuff.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1412,10 +1409,10 @@
         <v>10.11</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>13.56</v>
+        <v>13.8</v>
       </c>
       <c r="Y7" t="n">
-        <v>33.56</v>
+        <v>33.8</v>
       </c>
       <c r="Z7" t="n">
         <v>43.99</v>
@@ -1437,51 +1434,51 @@
       </c>
       <c r="AI7" t="inlineStr">
         <is>
-          <t>Same CJ product as S01: unbranded EVA garden clog with plush lining; lacks the Crocs furry exterior and strap; no closer furry-lined clog found on CJ.</t>
+          <t>Unbranded plush-lined garden clog mule (closed toe, fuzzy lining) rather than Crocs Cozzzy open sandal-slipper; listed as men's/couple sizes 36-45.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>A11</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Shoes</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>The Barb Wire Choker Danielle Guizio X The M Jewelers Necklace</t>
+          <t>Crocs Adult Unfurgettable Furry Lined Clogs, Fuzzy Slippers</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>87038.5</v>
+        <v>238816.09</v>
       </c>
       <c r="F8" t="n">
-        <v>1238</v>
+        <v>5002</v>
       </c>
       <c r="G8" t="n">
-        <v>70.31</v>
+        <v>47.74</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>-10.01</t>
+          <t>58.31</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>themjewelersny</t>
+          <t>CROCS US SHOP</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/view/product/1732377057880544126?region=US</t>
+          <t>https://www.tiktok.com/view/product/1732481650106799038?region=US</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1491,34 +1488,34 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>no</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Barbed-wire idea matches but CJ is a chunky silver iced-out chain; the winner is a dainty gold choker. CJ cost $26.</t>
+          <t>Winner is a fur-covered clog; CJ is a perforated garden clog with a fur cuff.</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2.5mm Wire Chain Hip Hop Necklace Micro Inlaid Sun Word Buckle Thorns</t>
+          <t>Fuzzy Plush Garden Clogs Mules Slippers Home Indoor Couple Slippers</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>CJLX1518256</t>
+          <t>CJNS1050784</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>https://www.cjdropshipping.com/product/2.5mm-wire-chain-hip-hop-necklace-micro-inlaid-sun-word-buckle-thorns-p-1544546445079498752.html</t>
+          <t>https://www.cjdropshipping.com/product/fuzzy-plush-garden-clogs-mules-slippers-home-indoor-couple-slippers-p-1373889976009363456.html</t>
         </is>
       </c>
       <c r="Q8" t="n">
-        <v>26.41</v>
+        <v>2.3</v>
       </c>
       <c r="R8" t="n">
-        <v>42</v>
+        <v>269</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1526,51 +1523,48 @@
         </is>
       </c>
       <c r="T8" t="n">
-        <v>5.01</v>
+        <v>7.81</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>CJPacket Pure Electricity</t>
+          <t>LuWei Ordinary US</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>7-14</t>
+          <t>5-11</t>
         </is>
       </c>
       <c r="W8" t="n">
-        <v>31.42</v>
+        <v>10.11</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>13.04</v>
+        <v>13.56</v>
       </c>
       <c r="Y8" t="n">
-        <v>33.04</v>
+        <v>33.56</v>
       </c>
       <c r="Z8" t="n">
-        <v>67.99000000000001</v>
+        <v>43.99</v>
       </c>
       <c r="AA8" t="n">
-        <v>-3</v>
+        <v>-8</v>
       </c>
       <c r="AB8" t="b">
         <v>1</v>
       </c>
       <c r="AC8" t="n">
-        <v>14</v>
+        <v>543</v>
       </c>
       <c r="AD8" t="n">
-        <v>192925</v>
-      </c>
-      <c r="AE8" t="n">
-        <v>0</v>
+        <v>2000000</v>
       </c>
       <c r="AF8" t="n">
         <v>0</v>
       </c>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>Unbranded lookalike: thin 2.5mm micro-pave CZ barbed-wire chain on gold-plated copper (gold/white gold, 14-20in), not the Danielle Guizio x M Jewelers piece; cost is high for CJ.</t>
+          <t>Same CJ product as S01: unbranded EVA garden clog with plush lining; lacks the Crocs furry exterior and strap; no closer furry-lined clog found on CJ.</t>
         </is>
       </c>
     </row>

</xml_diff>